<commit_message>
Receipt printers (ESC/POS and text) with downloads on the receipt page, Excel charts, JasperReports export and import, lower memory for large reports, limitations updated; 0.4.2 in the version history
</commit_message>
<xml_diff>
--- a/previews/laba-rugi.xlsx
+++ b/previews/laba-rugi.xlsx
@@ -124,6 +124,296 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4E79A7"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="2"/>
+              <c:pt idx="0">
+                <c:v>Pendapatan</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>Beban</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numLit>
+              <c:formatCode>General</c:formatCode>
+              <c:ptCount val="2"/>
+              <c:pt idx="0">
+                <c:v>72550000</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>53150000</c:v>
+              </c:pt>
+            </c:numLit>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:tickLblPos val="low"/>
+        <c:crossAx val="2"/>
+        <c:crosses val="autoZero"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4E79A7"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="F28E2B"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="76B7B2"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="59A14F"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="EDC948"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="6"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="B07AA1"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="7"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="9C755F"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="8"/>
+              <c:pt idx="0">
+                <c:v>Penjualan minuman</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>Penjualan makanan</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>Pesanan katering</c:v>
+              </c:pt>
+              <c:pt idx="3">
+                <c:v>Bahan baku</c:v>
+              </c:pt>
+              <c:pt idx="4">
+                <c:v>Gaji karyawan</c:v>
+              </c:pt>
+              <c:pt idx="5">
+                <c:v>Sewa tempat</c:v>
+              </c:pt>
+              <c:pt idx="6">
+                <c:v>Listrik dan air</c:v>
+              </c:pt>
+              <c:pt idx="7">
+                <c:v>Pemasaran</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numLit>
+              <c:formatCode>General</c:formatCode>
+              <c:ptCount val="8"/>
+              <c:pt idx="0">
+                <c:v>0</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>0</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>0</c:v>
+              </c:pt>
+              <c:pt idx="3">
+                <c:v>24300000</c:v>
+              </c:pt>
+              <c:pt idx="4">
+                <c:v>18000000</c:v>
+              </c:pt>
+              <c:pt idx="5">
+                <c:v>7500000</c:v>
+              </c:pt>
+              <c:pt idx="6">
+                <c:v>2150000</c:v>
+              </c:pt>
+              <c:pt idx="7">
+                <c:v>1200000</c:v>
+              </c:pt>
+            </c:numLit>
+          </c:val>
+        </c:ser>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="50"/>
+      </c:doughnutChart>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3175000" cy="2032000"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="3175000" cy="2032000"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>3187700</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3175000" cy="2032000"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="3175000" cy="2032000"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
@@ -259,7 +549,7 @@
         <v>53150000</v>
       </c>
     </row>
-    <row>
+    <row ht="160.0" customHeight="1">
       <c s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">LABA BERSIH</t>
@@ -278,5 +568,6 @@
       <c/>
     </row>
   </sheetData>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>